<commit_message>
Add placeholder village descriptions
</commit_message>
<xml_diff>
--- a/greece-dance/content/atlas.xlsx
+++ b/greece-dance/content/atlas.xlsx
@@ -126,10 +126,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -161,10 +161,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -404,18 +404,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L43"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="11.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="60.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="11.83203125" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="20.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="11.83203125"/>
+    <col min="4" max="4" customWidth="1" width="24.83203125"/>
+    <col min="5" max="5" customWidth="1" width="20.83203125"/>
+    <col min="6" max="6" customWidth="1" width="12.83203125"/>
+    <col min="7" max="7" customWidth="1" width="22.83203125"/>
+    <col min="8" max="8" customWidth="1" width="18.83203125"/>
+    <col min="9" max="9" customWidth="1" width="60.83203125"/>
+    <col min="10" max="10" customWidth="1" width="10.83203125"/>
+    <col min="11" max="11" customWidth="1" width="11.83203125"/>
+    <col min="12" max="12" customWidth="1" width="10.83203125"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -456,7 +456,7 @@
         <v>priority</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
         <v>bana</v>
       </c>
@@ -481,8 +481,9 @@
       <c r="H2" t="str">
         <v/>
       </c>
-      <c r="I2" t="str">
-        <v/>
+      <c r="I2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J2" t="str">
         <v>village</v>
@@ -494,7 +495,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" xml:space="preserve">
       <c r="A3" t="str">
         <v>boyialiki</v>
       </c>
@@ -519,8 +520,9 @@
       <c r="H3" t="str">
         <v/>
       </c>
-      <c r="I3" t="str">
-        <v/>
+      <c r="I3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J3" t="str">
         <v>village</v>
@@ -532,7 +534,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" xml:space="preserve">
       <c r="A4" t="str">
         <v>kavakli</v>
       </c>
@@ -557,8 +559,9 @@
       <c r="H4" t="str">
         <v/>
       </c>
-      <c r="I4" t="str">
-        <v/>
+      <c r="I4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J4" t="str">
         <v>village</v>
@@ -570,7 +573,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" xml:space="preserve">
       <c r="A5" t="str">
         <v>asvestades</v>
       </c>
@@ -595,8 +598,9 @@
       <c r="H5" t="str">
         <v/>
       </c>
-      <c r="I5" t="str">
-        <v/>
+      <c r="I5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J5" t="str">
         <v>village</v>
@@ -608,7 +612,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" xml:space="preserve">
       <c r="A6" t="str">
         <v>metaxades</v>
       </c>
@@ -633,8 +637,9 @@
       <c r="H6" t="str">
         <v/>
       </c>
-      <c r="I6" t="str">
-        <v/>
+      <c r="I6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J6" t="str">
         <v>village</v>
@@ -646,7 +651,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" xml:space="preserve">
       <c r="A7" t="str">
         <v>serres</v>
       </c>
@@ -671,8 +676,9 @@
       <c r="H7" t="str">
         <v/>
       </c>
-      <c r="I7" t="str">
-        <v/>
+      <c r="I7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J7" t="str">
         <v>city</v>
@@ -684,7 +690,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" xml:space="preserve">
       <c r="A8" t="str">
         <v>drama</v>
       </c>
@@ -709,8 +715,9 @@
       <c r="H8" t="str">
         <v/>
       </c>
-      <c r="I8" t="str">
-        <v/>
+      <c r="I8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J8" t="str">
         <v>city</v>
@@ -722,7 +729,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" xml:space="preserve">
       <c r="A9" t="str">
         <v>pylaia</v>
       </c>
@@ -747,8 +754,9 @@
       <c r="H9" t="str">
         <v/>
       </c>
-      <c r="I9" t="str">
-        <v/>
+      <c r="I9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J9" t="str">
         <v>town</v>
@@ -760,7 +768,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" xml:space="preserve">
       <c r="A10" t="str">
         <v>aridaia</v>
       </c>
@@ -785,8 +793,9 @@
       <c r="H10" t="str">
         <v/>
       </c>
-      <c r="I10" t="str">
-        <v/>
+      <c r="I10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J10" t="str">
         <v>town</v>
@@ -798,7 +807,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" xml:space="preserve">
       <c r="A11" t="str">
         <v>edessa</v>
       </c>
@@ -823,8 +832,9 @@
       <c r="H11" t="str">
         <v/>
       </c>
-      <c r="I11" t="str">
-        <v/>
+      <c r="I11" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J11" t="str">
         <v>town</v>
@@ -836,7 +846,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" xml:space="preserve">
       <c r="A12" t="str">
         <v>promarhoi</v>
       </c>
@@ -861,8 +871,9 @@
       <c r="H12" t="str">
         <v/>
       </c>
-      <c r="I12" t="str">
-        <v/>
+      <c r="I12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J12" t="str">
         <v>village</v>
@@ -874,7 +885,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" xml:space="preserve">
       <c r="A13" t="str">
         <v>orma</v>
       </c>
@@ -899,8 +910,9 @@
       <c r="H13" t="str">
         <v/>
       </c>
-      <c r="I13" t="str">
-        <v/>
+      <c r="I13" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J13" t="str">
         <v>village</v>
@@ -912,7 +924,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" xml:space="preserve">
       <c r="A14" t="str">
         <v>karydia</v>
       </c>
@@ -937,8 +949,9 @@
       <c r="H14" t="str">
         <v/>
       </c>
-      <c r="I14" t="str">
-        <v/>
+      <c r="I14" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J14" t="str">
         <v>village</v>
@@ -950,7 +963,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" xml:space="preserve">
       <c r="A15" t="str">
         <v>arnissa</v>
       </c>
@@ -975,8 +988,9 @@
       <c r="H15" t="str">
         <v/>
       </c>
-      <c r="I15" t="str">
-        <v/>
+      <c r="I15" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J15" t="str">
         <v>village</v>
@@ -988,7 +1002,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" xml:space="preserve">
       <c r="A16" t="str">
         <v>goumenissa</v>
       </c>
@@ -1013,8 +1027,9 @@
       <c r="H16" t="str">
         <v/>
       </c>
-      <c r="I16" t="str">
-        <v/>
+      <c r="I16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J16" t="str">
         <v>town</v>
@@ -1026,7 +1041,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" xml:space="preserve">
       <c r="A17" t="str">
         <v>naoussa</v>
       </c>
@@ -1051,8 +1066,9 @@
       <c r="H17" t="str">
         <v/>
       </c>
-      <c r="I17" t="str">
-        <v/>
+      <c r="I17" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J17" t="str">
         <v>town</v>
@@ -1064,7 +1080,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" xml:space="preserve">
       <c r="A18" t="str">
         <v>roumlouki</v>
       </c>
@@ -1089,8 +1105,9 @@
       <c r="H18" t="str">
         <v/>
       </c>
-      <c r="I18" t="str">
-        <v/>
+      <c r="I18" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J18" t="str">
         <v>village</v>
@@ -1102,7 +1119,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" xml:space="preserve">
       <c r="A19" t="str">
         <v>florina</v>
       </c>
@@ -1127,8 +1144,9 @@
       <c r="H19" t="str">
         <v/>
       </c>
-      <c r="I19" t="str">
-        <v/>
+      <c r="I19" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J19" t="str">
         <v>city</v>
@@ -1140,7 +1158,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" xml:space="preserve">
       <c r="A20" t="str">
         <v>kastoria</v>
       </c>
@@ -1165,8 +1183,9 @@
       <c r="H20" t="str">
         <v/>
       </c>
-      <c r="I20" t="str">
-        <v/>
+      <c r="I20" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J20" t="str">
         <v>city</v>
@@ -1178,7 +1197,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" xml:space="preserve">
       <c r="A21" t="str">
         <v>grevena</v>
       </c>
@@ -1203,8 +1222,9 @@
       <c r="H21" t="str">
         <v/>
       </c>
-      <c r="I21" t="str">
-        <v/>
+      <c r="I21" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J21" t="str">
         <v>city</v>
@@ -1216,7 +1236,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" xml:space="preserve">
       <c r="A22" t="str">
         <v>deskati</v>
       </c>
@@ -1241,8 +1261,9 @@
       <c r="H22" t="str">
         <v/>
       </c>
-      <c r="I22" t="str">
-        <v/>
+      <c r="I22" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J22" t="str">
         <v>town</v>
@@ -1254,7 +1275,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" xml:space="preserve">
       <c r="A23" t="str">
         <v>megara</v>
       </c>
@@ -1279,8 +1300,9 @@
       <c r="H23" t="str">
         <v/>
       </c>
-      <c r="I23" t="str">
-        <v/>
+      <c r="I23" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J23" t="str">
         <v>city</v>
@@ -1292,7 +1314,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" xml:space="preserve">
       <c r="A24" t="str">
         <v>salamina</v>
       </c>
@@ -1317,8 +1339,9 @@
       <c r="H24" t="str">
         <v/>
       </c>
-      <c r="I24" t="str">
-        <v/>
+      <c r="I24" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J24" t="str">
         <v>town</v>
@@ -1330,7 +1353,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" xml:space="preserve">
       <c r="A25" t="str">
         <v>argithea</v>
       </c>
@@ -1355,8 +1378,9 @@
       <c r="H25" t="str">
         <v>Agrafa</v>
       </c>
-      <c r="I25" t="str">
-        <v/>
+      <c r="I25" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J25" t="str">
         <v>village</v>
@@ -1368,7 +1392,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" xml:space="preserve">
       <c r="A26" t="str">
         <v>krioneri</v>
       </c>
@@ -1393,8 +1417,9 @@
       <c r="H26" t="str">
         <v>Agrafa</v>
       </c>
-      <c r="I26" t="str">
-        <v/>
+      <c r="I26" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J26" t="str">
         <v>village</v>
@@ -1406,7 +1431,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" xml:space="preserve">
       <c r="A27" t="str">
         <v>thrapsimi</v>
       </c>
@@ -1431,8 +1456,9 @@
       <c r="H27" t="str">
         <v>Agrafa</v>
       </c>
-      <c r="I27" t="str">
-        <v/>
+      <c r="I27" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J27" t="str">
         <v>village</v>
@@ -1444,7 +1470,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" xml:space="preserve">
       <c r="A28" t="str">
         <v>sofades</v>
       </c>
@@ -1469,8 +1495,9 @@
       <c r="H28" t="str">
         <v/>
       </c>
-      <c r="I28" t="str">
-        <v/>
+      <c r="I28" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J28" t="str">
         <v>town</v>
@@ -1482,7 +1509,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" xml:space="preserve">
       <c r="A29" t="str">
         <v>rizomata</v>
       </c>
@@ -1507,8 +1534,9 @@
       <c r="H29" t="str">
         <v/>
       </c>
-      <c r="I29" t="str">
-        <v/>
+      <c r="I29" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J29" t="str">
         <v>village</v>
@@ -1520,7 +1548,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" xml:space="preserve">
       <c r="A30" t="str">
         <v>elatohori</v>
       </c>
@@ -1545,8 +1573,9 @@
       <c r="H30" t="str">
         <v/>
       </c>
-      <c r="I30" t="str">
-        <v/>
+      <c r="I30" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J30" t="str">
         <v>village</v>
@@ -1558,7 +1587,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" xml:space="preserve">
       <c r="A31" t="str">
         <v>toxo</v>
       </c>
@@ -1583,8 +1612,9 @@
       <c r="H31" t="str">
         <v/>
       </c>
-      <c r="I31" t="str">
-        <v/>
+      <c r="I31" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J31" t="str">
         <v>village</v>
@@ -1596,7 +1626,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" xml:space="preserve">
       <c r="A32" t="str">
         <v>dion</v>
       </c>
@@ -1621,8 +1651,9 @@
       <c r="H32" t="str">
         <v/>
       </c>
-      <c r="I32" t="str">
-        <v/>
+      <c r="I32" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J32" t="str">
         <v>village</v>
@@ -1634,7 +1665,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" xml:space="preserve">
       <c r="A33" t="str">
         <v>vrontou</v>
       </c>
@@ -1659,8 +1690,9 @@
       <c r="H33" t="str">
         <v/>
       </c>
-      <c r="I33" t="str">
-        <v/>
+      <c r="I33" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J33" t="str">
         <v>village</v>
@@ -1672,7 +1704,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" xml:space="preserve">
       <c r="A34" t="str">
         <v>kefallonia</v>
       </c>
@@ -1697,8 +1729,9 @@
       <c r="H34" t="str">
         <v/>
       </c>
-      <c r="I34" t="str">
-        <v/>
+      <c r="I34" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J34" t="str">
         <v>village</v>
@@ -1710,7 +1743,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" xml:space="preserve">
       <c r="A35" t="str">
         <v>kerkyra</v>
       </c>
@@ -1735,8 +1768,9 @@
       <c r="H35" t="str">
         <v/>
       </c>
-      <c r="I35" t="str">
-        <v/>
+      <c r="I35" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J35" t="str">
         <v>village</v>
@@ -1748,7 +1782,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" xml:space="preserve">
       <c r="A36" t="str">
         <v>zakinthos</v>
       </c>
@@ -1773,8 +1807,9 @@
       <c r="H36" t="str">
         <v/>
       </c>
-      <c r="I36" t="str">
-        <v/>
+      <c r="I36" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J36" t="str">
         <v>village</v>
@@ -1786,7 +1821,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" xml:space="preserve">
       <c r="A37" t="str">
         <v>naxos</v>
       </c>
@@ -1811,8 +1846,9 @@
       <c r="H37" t="str">
         <v/>
       </c>
-      <c r="I37" t="str">
-        <v/>
+      <c r="I37" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J37" t="str">
         <v>village</v>
@@ -1824,7 +1860,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" xml:space="preserve">
       <c r="A38" t="str">
         <v>paros</v>
       </c>
@@ -1849,8 +1885,9 @@
       <c r="H38" t="str">
         <v/>
       </c>
-      <c r="I38" t="str">
-        <v/>
+      <c r="I38" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J38" t="str">
         <v>village</v>
@@ -1862,7 +1899,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" xml:space="preserve">
       <c r="A39" t="str">
         <v>ikaria</v>
       </c>
@@ -1887,8 +1924,9 @@
       <c r="H39" t="str">
         <v/>
       </c>
-      <c r="I39" t="str">
-        <v/>
+      <c r="I39" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J39" t="str">
         <v>village</v>
@@ -1900,7 +1938,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" xml:space="preserve">
       <c r="A40" t="str">
         <v>lesvos</v>
       </c>
@@ -1925,8 +1963,9 @@
       <c r="H40" t="str">
         <v/>
       </c>
-      <c r="I40" t="str">
-        <v/>
+      <c r="I40" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J40" t="str">
         <v>village</v>
@@ -1938,7 +1977,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" xml:space="preserve">
       <c r="A41" t="str">
         <v>hania</v>
       </c>
@@ -1963,8 +2002,9 @@
       <c r="H41" t="str">
         <v/>
       </c>
-      <c r="I41" t="str">
-        <v/>
+      <c r="I41" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J41" t="str">
         <v>city</v>
@@ -1976,7 +2016,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" xml:space="preserve">
       <c r="A42" t="str">
         <v>rethimno</v>
       </c>
@@ -2001,8 +2041,9 @@
       <c r="H42" t="str">
         <v/>
       </c>
-      <c r="I42" t="str">
-        <v/>
+      <c r="I42" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J42" t="str">
         <v>city</v>
@@ -2014,7 +2055,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" xml:space="preserve">
       <c r="A43" t="str">
         <v>alatsata</v>
       </c>
@@ -2039,8 +2080,9 @@
       <c r="H43" t="str">
         <v/>
       </c>
-      <c r="I43" t="str">
-        <v/>
+      <c r="I43" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.
+Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</v>
       </c>
       <c r="J43" t="str">
         <v>village</v>
@@ -2064,15 +2106,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I25"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="72.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="11.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="8.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="22.83203125"/>
+    <col min="2" max="2" customWidth="1" width="72.83203125"/>
+    <col min="3" max="3" customWidth="1" width="24.83203125"/>
+    <col min="4" max="4" customWidth="1" width="11.83203125"/>
+    <col min="5" max="5" customWidth="1" width="10.83203125"/>
+    <col min="6" max="6" customWidth="1" width="10.83203125"/>
+    <col min="7" max="7" customWidth="1" width="10.83203125"/>
+    <col min="8" max="8" customWidth="1" width="10.83203125"/>
+    <col min="9" max="9" customWidth="1" width="8.83203125"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Remove automatic map camera movement
</commit_message>
<xml_diff>
--- a/greece-dance/content/atlas.xlsx
+++ b/greece-dance/content/atlas.xlsx
@@ -8,7 +8,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">Places!$A$1:$L$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">Regions!$A$1:$I$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">Regions!$A$1:$E$25</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -2104,17 +2104,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:E25"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="22.83203125"/>
     <col min="2" max="2" customWidth="1" width="72.83203125"/>
     <col min="3" max="3" customWidth="1" width="24.83203125"/>
     <col min="4" max="4" customWidth="1" width="11.83203125"/>
-    <col min="5" max="5" customWidth="1" width="10.83203125"/>
-    <col min="6" max="6" customWidth="1" width="10.83203125"/>
-    <col min="7" max="7" customWidth="1" width="10.83203125"/>
-    <col min="8" max="8" customWidth="1" width="10.83203125"/>
-    <col min="9" max="9" customWidth="1" width="8.83203125"/>
+    <col min="5" max="5" customWidth="1" width="8.83203125"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2131,18 +2127,6 @@
         <v>color</v>
       </c>
       <c r="E1" t="str">
-        <v>south</v>
-      </c>
-      <c r="F1" t="str">
-        <v>west</v>
-      </c>
-      <c r="G1" t="str">
-        <v>north</v>
-      </c>
-      <c r="H1" t="str">
-        <v>east</v>
-      </c>
-      <c r="I1" t="str">
         <v>order</v>
       </c>
     </row>
@@ -2160,18 +2144,6 @@
         <v>#b85c4a</v>
       </c>
       <c r="E2">
-        <v>41.8</v>
-      </c>
-      <c r="F2">
-        <v>25.8</v>
-      </c>
-      <c r="G2">
-        <v>43.1</v>
-      </c>
-      <c r="H2">
-        <v>28.3</v>
-      </c>
-      <c r="I2">
         <v>1</v>
       </c>
     </row>
@@ -2189,18 +2161,6 @@
         <v>#4d8f83</v>
       </c>
       <c r="E3">
-        <v>41</v>
-      </c>
-      <c r="F3">
-        <v>25.8</v>
-      </c>
-      <c r="G3">
-        <v>41.7</v>
-      </c>
-      <c r="H3">
-        <v>26.8</v>
-      </c>
-      <c r="I3">
         <v>2</v>
       </c>
     </row>
@@ -2218,18 +2178,6 @@
         <v>#3f77a6</v>
       </c>
       <c r="E4">
-        <v>40.7</v>
-      </c>
-      <c r="F4">
-        <v>23.1</v>
-      </c>
-      <c r="G4">
-        <v>41.4</v>
-      </c>
-      <c r="H4">
-        <v>24.5</v>
-      </c>
-      <c r="I4">
         <v>3</v>
       </c>
     </row>
@@ -2247,18 +2195,6 @@
         <v>#a66b3f</v>
       </c>
       <c r="E5">
-        <v>40.3</v>
-      </c>
-      <c r="F5">
-        <v>22.5</v>
-      </c>
-      <c r="G5">
-        <v>40.9</v>
-      </c>
-      <c r="H5">
-        <v>23.4</v>
-      </c>
-      <c r="I5">
         <v>4</v>
       </c>
     </row>
@@ -2276,18 +2212,6 @@
         <v>#e5a83f</v>
       </c>
       <c r="E6">
-        <v>40.5</v>
-      </c>
-      <c r="F6">
-        <v>21.5</v>
-      </c>
-      <c r="G6">
-        <v>41.3</v>
-      </c>
-      <c r="H6">
-        <v>22.4</v>
-      </c>
-      <c r="I6">
         <v>5</v>
       </c>
     </row>
@@ -2305,18 +2229,6 @@
         <v>#6f8f4d</v>
       </c>
       <c r="E7">
-        <v>40.3</v>
-      </c>
-      <c r="F7">
-        <v>21.7</v>
-      </c>
-      <c r="G7">
-        <v>41.2</v>
-      </c>
-      <c r="H7">
-        <v>22.8</v>
-      </c>
-      <c r="I7">
         <v>6</v>
       </c>
     </row>
@@ -2334,18 +2246,6 @@
         <v>#7c6aaa</v>
       </c>
       <c r="E8">
-        <v>39.6</v>
-      </c>
-      <c r="F8">
-        <v>20.8</v>
-      </c>
-      <c r="G8">
-        <v>41.1</v>
-      </c>
-      <c r="H8">
-        <v>22.2</v>
-      </c>
-      <c r="I8">
         <v>7</v>
       </c>
     </row>
@@ -2363,18 +2263,6 @@
         <v>#ce5e33</v>
       </c>
       <c r="E9">
-        <v>37.6</v>
-      </c>
-      <c r="F9">
-        <v>22.8</v>
-      </c>
-      <c r="G9">
-        <v>38.3</v>
-      </c>
-      <c r="H9">
-        <v>24</v>
-      </c>
-      <c r="I9">
         <v>8</v>
       </c>
     </row>
@@ -2392,18 +2280,6 @@
         <v>#9b7554</v>
       </c>
       <c r="E10">
-        <v>36.3</v>
-      </c>
-      <c r="F10">
-        <v>21</v>
-      </c>
-      <c r="G10">
-        <v>38.5</v>
-      </c>
-      <c r="H10">
-        <v>23.6</v>
-      </c>
-      <c r="I10">
         <v>9</v>
       </c>
     </row>
@@ -2421,18 +2297,6 @@
         <v>#5f8f6e</v>
       </c>
       <c r="E11">
-        <v>38.8</v>
-      </c>
-      <c r="F11">
-        <v>21</v>
-      </c>
-      <c r="G11">
-        <v>40</v>
-      </c>
-      <c r="H11">
-        <v>23</v>
-      </c>
-      <c r="I11">
         <v>10</v>
       </c>
     </row>
@@ -2450,18 +2314,6 @@
         <v>#bf7b4a</v>
       </c>
       <c r="E12">
-        <v>39.9</v>
-      </c>
-      <c r="F12">
-        <v>21.9</v>
-      </c>
-      <c r="G12">
-        <v>40.6</v>
-      </c>
-      <c r="H12">
-        <v>22.8</v>
-      </c>
-      <c r="I12">
         <v>11</v>
       </c>
     </row>
@@ -2479,18 +2331,6 @@
         <v>#667d5e</v>
       </c>
       <c r="E13">
-        <v>38.7</v>
-      </c>
-      <c r="F13">
-        <v>19.7</v>
-      </c>
-      <c r="G13">
-        <v>40.4</v>
-      </c>
-      <c r="H13">
-        <v>21.6</v>
-      </c>
-      <c r="I13">
         <v>12</v>
       </c>
     </row>
@@ -2508,18 +2348,6 @@
         <v>#8a6d5b</v>
       </c>
       <c r="E14">
-        <v>38.5</v>
-      </c>
-      <c r="F14">
-        <v>20</v>
-      </c>
-      <c r="G14">
-        <v>41.5</v>
-      </c>
-      <c r="H14">
-        <v>24.5</v>
-      </c>
-      <c r="I14">
         <v>13</v>
       </c>
     </row>
@@ -2537,18 +2365,6 @@
         <v>#4f8b86</v>
       </c>
       <c r="E15">
-        <v>37.9</v>
-      </c>
-      <c r="F15">
-        <v>22.8</v>
-      </c>
-      <c r="G15">
-        <v>39.1</v>
-      </c>
-      <c r="H15">
-        <v>24.6</v>
-      </c>
-      <c r="I15">
         <v>14</v>
       </c>
     </row>
@@ -2566,18 +2382,6 @@
         <v>#4b78a2</v>
       </c>
       <c r="E16">
-        <v>37.5</v>
-      </c>
-      <c r="F16">
-        <v>19.3</v>
-      </c>
-      <c r="G16">
-        <v>39.9</v>
-      </c>
-      <c r="H16">
-        <v>21.3</v>
-      </c>
-      <c r="I16">
         <v>15</v>
       </c>
     </row>
@@ -2595,18 +2399,6 @@
         <v>#5d8fad</v>
       </c>
       <c r="E17">
-        <v>36.2</v>
-      </c>
-      <c r="F17">
-        <v>24.2</v>
-      </c>
-      <c r="G17">
-        <v>38</v>
-      </c>
-      <c r="H17">
-        <v>27</v>
-      </c>
-      <c r="I17">
         <v>16</v>
       </c>
     </row>
@@ -2624,18 +2416,6 @@
         <v>#3f8778</v>
       </c>
       <c r="E18">
-        <v>38.9</v>
-      </c>
-      <c r="F18">
-        <v>22.7</v>
-      </c>
-      <c r="G18">
-        <v>39.4</v>
-      </c>
-      <c r="H18">
-        <v>24.4</v>
-      </c>
-      <c r="I18">
         <v>17</v>
       </c>
     </row>
@@ -2653,18 +2433,6 @@
         <v>#566eaa</v>
       </c>
       <c r="E19">
-        <v>38.8</v>
-      </c>
-      <c r="F19">
-        <v>25.7</v>
-      </c>
-      <c r="G19">
-        <v>39.5</v>
-      </c>
-      <c r="H19">
-        <v>26.7</v>
-      </c>
-      <c r="I19">
         <v>18</v>
       </c>
     </row>
@@ -2682,18 +2450,6 @@
         <v>#8b6bb3</v>
       </c>
       <c r="E20">
-        <v>35.3</v>
-      </c>
-      <c r="F20">
-        <v>26</v>
-      </c>
-      <c r="G20">
-        <v>37.6</v>
-      </c>
-      <c r="H20">
-        <v>29.8</v>
-      </c>
-      <c r="I20">
         <v>19</v>
       </c>
     </row>
@@ -2711,18 +2467,6 @@
         <v>#c45f45</v>
       </c>
       <c r="E21">
-        <v>34.7</v>
-      </c>
-      <c r="F21">
-        <v>23.3</v>
-      </c>
-      <c r="G21">
-        <v>35.7</v>
-      </c>
-      <c r="H21">
-        <v>26.5</v>
-      </c>
-      <c r="I21">
         <v>20</v>
       </c>
     </row>
@@ -2740,18 +2484,6 @@
         <v>#ad7f32</v>
       </c>
       <c r="E22">
-        <v>34.5</v>
-      </c>
-      <c r="F22">
-        <v>32.2</v>
-      </c>
-      <c r="G22">
-        <v>35.8</v>
-      </c>
-      <c r="H22">
-        <v>34.7</v>
-      </c>
-      <c r="I22">
         <v>21</v>
       </c>
     </row>
@@ -2769,18 +2501,6 @@
         <v>#ce5f83</v>
       </c>
       <c r="E23">
-        <v>36</v>
-      </c>
-      <c r="F23">
-        <v>25.8</v>
-      </c>
-      <c r="G23">
-        <v>41.2</v>
-      </c>
-      <c r="H23">
-        <v>30</v>
-      </c>
-      <c r="I23">
         <v>22</v>
       </c>
     </row>
@@ -2798,18 +2518,6 @@
         <v>#9a6e4f</v>
       </c>
       <c r="E24">
-        <v>37.5</v>
-      </c>
-      <c r="F24">
-        <v>32.5</v>
-      </c>
-      <c r="G24">
-        <v>39.8</v>
-      </c>
-      <c r="H24">
-        <v>36.5</v>
-      </c>
-      <c r="I24">
         <v>23</v>
       </c>
     </row>
@@ -2827,23 +2535,11 @@
         <v>#65758f</v>
       </c>
       <c r="E25">
-        <v>39.5</v>
-      </c>
-      <c r="F25">
-        <v>34</v>
-      </c>
-      <c r="G25">
-        <v>42.5</v>
-      </c>
-      <c r="H25">
-        <v>41.5</v>
-      </c>
-      <c r="I25">
         <v>24</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I25"/>
+  <autoFilter ref="A1:E25"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:I25"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
Move map labels to collision-aware overlay
</commit_message>
<xml_diff>
--- a/greece-dance/content/atlas.xlsx
+++ b/greece-dance/content/atlas.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Regions" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Places!$A$1:$L$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Places!$A$1:$J$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">Regions!$A$1:$E$25</definedName>
   </definedNames>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:J43"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="20.83203125"/>
     <col min="2" max="2" customWidth="1" width="11.83203125"/>
@@ -414,8 +414,6 @@
     <col min="8" max="8" customWidth="1" width="18.83203125"/>
     <col min="9" max="9" customWidth="1" width="60.83203125"/>
     <col min="10" max="10" customWidth="1" width="10.83203125"/>
-    <col min="11" max="11" customWidth="1" width="11.83203125"/>
-    <col min="12" max="12" customWidth="1" width="10.83203125"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,12 +447,6 @@
       <c r="J1" t="str">
         <v>kind</v>
       </c>
-      <c r="K1" t="str">
-        <v>min_zoom</v>
-      </c>
-      <c r="L1" t="str">
-        <v>priority</v>
-      </c>
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
@@ -488,12 +480,6 @@
       <c r="J2" t="str">
         <v>village</v>
       </c>
-      <c r="K2">
-        <v>8</v>
-      </c>
-      <c r="L2">
-        <v>600</v>
-      </c>
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
@@ -527,12 +513,6 @@
       <c r="J3" t="str">
         <v>village</v>
       </c>
-      <c r="K3">
-        <v>8</v>
-      </c>
-      <c r="L3">
-        <v>600</v>
-      </c>
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4" t="str">
@@ -566,12 +546,6 @@
       <c r="J4" t="str">
         <v>village</v>
       </c>
-      <c r="K4">
-        <v>8</v>
-      </c>
-      <c r="L4">
-        <v>600</v>
-      </c>
     </row>
     <row r="5" xml:space="preserve">
       <c r="A5" t="str">
@@ -605,12 +579,6 @@
       <c r="J5" t="str">
         <v>village</v>
       </c>
-      <c r="K5">
-        <v>8</v>
-      </c>
-      <c r="L5">
-        <v>600</v>
-      </c>
     </row>
     <row r="6" xml:space="preserve">
       <c r="A6" t="str">
@@ -644,12 +612,6 @@
       <c r="J6" t="str">
         <v>village</v>
       </c>
-      <c r="K6">
-        <v>8</v>
-      </c>
-      <c r="L6">
-        <v>600</v>
-      </c>
     </row>
     <row r="7" xml:space="preserve">
       <c r="A7" t="str">
@@ -683,12 +645,6 @@
       <c r="J7" t="str">
         <v>city</v>
       </c>
-      <c r="K7">
-        <v>6</v>
-      </c>
-      <c r="L7">
-        <v>900</v>
-      </c>
     </row>
     <row r="8" xml:space="preserve">
       <c r="A8" t="str">
@@ -722,12 +678,6 @@
       <c r="J8" t="str">
         <v>city</v>
       </c>
-      <c r="K8">
-        <v>6</v>
-      </c>
-      <c r="L8">
-        <v>900</v>
-      </c>
     </row>
     <row r="9" xml:space="preserve">
       <c r="A9" t="str">
@@ -761,12 +711,6 @@
       <c r="J9" t="str">
         <v>town</v>
       </c>
-      <c r="K9">
-        <v>7</v>
-      </c>
-      <c r="L9">
-        <v>750</v>
-      </c>
     </row>
     <row r="10" xml:space="preserve">
       <c r="A10" t="str">
@@ -800,12 +744,6 @@
       <c r="J10" t="str">
         <v>town</v>
       </c>
-      <c r="K10">
-        <v>7</v>
-      </c>
-      <c r="L10">
-        <v>750</v>
-      </c>
     </row>
     <row r="11" xml:space="preserve">
       <c r="A11" t="str">
@@ -839,12 +777,6 @@
       <c r="J11" t="str">
         <v>town</v>
       </c>
-      <c r="K11">
-        <v>7</v>
-      </c>
-      <c r="L11">
-        <v>750</v>
-      </c>
     </row>
     <row r="12" xml:space="preserve">
       <c r="A12" t="str">
@@ -878,12 +810,6 @@
       <c r="J12" t="str">
         <v>village</v>
       </c>
-      <c r="K12">
-        <v>8</v>
-      </c>
-      <c r="L12">
-        <v>600</v>
-      </c>
     </row>
     <row r="13" xml:space="preserve">
       <c r="A13" t="str">
@@ -917,12 +843,6 @@
       <c r="J13" t="str">
         <v>village</v>
       </c>
-      <c r="K13">
-        <v>8</v>
-      </c>
-      <c r="L13">
-        <v>600</v>
-      </c>
     </row>
     <row r="14" xml:space="preserve">
       <c r="A14" t="str">
@@ -956,12 +876,6 @@
       <c r="J14" t="str">
         <v>village</v>
       </c>
-      <c r="K14">
-        <v>8</v>
-      </c>
-      <c r="L14">
-        <v>600</v>
-      </c>
     </row>
     <row r="15" xml:space="preserve">
       <c r="A15" t="str">
@@ -995,12 +909,6 @@
       <c r="J15" t="str">
         <v>village</v>
       </c>
-      <c r="K15">
-        <v>8</v>
-      </c>
-      <c r="L15">
-        <v>600</v>
-      </c>
     </row>
     <row r="16" xml:space="preserve">
       <c r="A16" t="str">
@@ -1034,12 +942,6 @@
       <c r="J16" t="str">
         <v>town</v>
       </c>
-      <c r="K16">
-        <v>7</v>
-      </c>
-      <c r="L16">
-        <v>750</v>
-      </c>
     </row>
     <row r="17" xml:space="preserve">
       <c r="A17" t="str">
@@ -1073,12 +975,6 @@
       <c r="J17" t="str">
         <v>town</v>
       </c>
-      <c r="K17">
-        <v>7</v>
-      </c>
-      <c r="L17">
-        <v>750</v>
-      </c>
     </row>
     <row r="18" xml:space="preserve">
       <c r="A18" t="str">
@@ -1112,12 +1008,6 @@
       <c r="J18" t="str">
         <v>village</v>
       </c>
-      <c r="K18">
-        <v>8</v>
-      </c>
-      <c r="L18">
-        <v>600</v>
-      </c>
     </row>
     <row r="19" xml:space="preserve">
       <c r="A19" t="str">
@@ -1151,12 +1041,6 @@
       <c r="J19" t="str">
         <v>city</v>
       </c>
-      <c r="K19">
-        <v>6</v>
-      </c>
-      <c r="L19">
-        <v>900</v>
-      </c>
     </row>
     <row r="20" xml:space="preserve">
       <c r="A20" t="str">
@@ -1190,12 +1074,6 @@
       <c r="J20" t="str">
         <v>city</v>
       </c>
-      <c r="K20">
-        <v>6</v>
-      </c>
-      <c r="L20">
-        <v>900</v>
-      </c>
     </row>
     <row r="21" xml:space="preserve">
       <c r="A21" t="str">
@@ -1229,12 +1107,6 @@
       <c r="J21" t="str">
         <v>city</v>
       </c>
-      <c r="K21">
-        <v>6</v>
-      </c>
-      <c r="L21">
-        <v>900</v>
-      </c>
     </row>
     <row r="22" xml:space="preserve">
       <c r="A22" t="str">
@@ -1268,12 +1140,6 @@
       <c r="J22" t="str">
         <v>town</v>
       </c>
-      <c r="K22">
-        <v>7</v>
-      </c>
-      <c r="L22">
-        <v>750</v>
-      </c>
     </row>
     <row r="23" xml:space="preserve">
       <c r="A23" t="str">
@@ -1307,12 +1173,6 @@
       <c r="J23" t="str">
         <v>city</v>
       </c>
-      <c r="K23">
-        <v>6</v>
-      </c>
-      <c r="L23">
-        <v>900</v>
-      </c>
     </row>
     <row r="24" xml:space="preserve">
       <c r="A24" t="str">
@@ -1346,12 +1206,6 @@
       <c r="J24" t="str">
         <v>town</v>
       </c>
-      <c r="K24">
-        <v>7</v>
-      </c>
-      <c r="L24">
-        <v>750</v>
-      </c>
     </row>
     <row r="25" xml:space="preserve">
       <c r="A25" t="str">
@@ -1385,12 +1239,6 @@
       <c r="J25" t="str">
         <v>village</v>
       </c>
-      <c r="K25">
-        <v>8</v>
-      </c>
-      <c r="L25">
-        <v>600</v>
-      </c>
     </row>
     <row r="26" xml:space="preserve">
       <c r="A26" t="str">
@@ -1424,12 +1272,6 @@
       <c r="J26" t="str">
         <v>village</v>
       </c>
-      <c r="K26">
-        <v>8</v>
-      </c>
-      <c r="L26">
-        <v>600</v>
-      </c>
     </row>
     <row r="27" xml:space="preserve">
       <c r="A27" t="str">
@@ -1463,12 +1305,6 @@
       <c r="J27" t="str">
         <v>village</v>
       </c>
-      <c r="K27">
-        <v>8</v>
-      </c>
-      <c r="L27">
-        <v>600</v>
-      </c>
     </row>
     <row r="28" xml:space="preserve">
       <c r="A28" t="str">
@@ -1502,12 +1338,6 @@
       <c r="J28" t="str">
         <v>town</v>
       </c>
-      <c r="K28">
-        <v>7</v>
-      </c>
-      <c r="L28">
-        <v>750</v>
-      </c>
     </row>
     <row r="29" xml:space="preserve">
       <c r="A29" t="str">
@@ -1541,12 +1371,6 @@
       <c r="J29" t="str">
         <v>village</v>
       </c>
-      <c r="K29">
-        <v>8</v>
-      </c>
-      <c r="L29">
-        <v>600</v>
-      </c>
     </row>
     <row r="30" xml:space="preserve">
       <c r="A30" t="str">
@@ -1580,12 +1404,6 @@
       <c r="J30" t="str">
         <v>village</v>
       </c>
-      <c r="K30">
-        <v>8</v>
-      </c>
-      <c r="L30">
-        <v>600</v>
-      </c>
     </row>
     <row r="31" xml:space="preserve">
       <c r="A31" t="str">
@@ -1619,12 +1437,6 @@
       <c r="J31" t="str">
         <v>village</v>
       </c>
-      <c r="K31">
-        <v>8</v>
-      </c>
-      <c r="L31">
-        <v>600</v>
-      </c>
     </row>
     <row r="32" xml:space="preserve">
       <c r="A32" t="str">
@@ -1658,12 +1470,6 @@
       <c r="J32" t="str">
         <v>village</v>
       </c>
-      <c r="K32">
-        <v>8</v>
-      </c>
-      <c r="L32">
-        <v>600</v>
-      </c>
     </row>
     <row r="33" xml:space="preserve">
       <c r="A33" t="str">
@@ -1697,12 +1503,6 @@
       <c r="J33" t="str">
         <v>village</v>
       </c>
-      <c r="K33">
-        <v>8</v>
-      </c>
-      <c r="L33">
-        <v>600</v>
-      </c>
     </row>
     <row r="34" xml:space="preserve">
       <c r="A34" t="str">
@@ -1736,12 +1536,6 @@
       <c r="J34" t="str">
         <v>village</v>
       </c>
-      <c r="K34">
-        <v>8</v>
-      </c>
-      <c r="L34">
-        <v>600</v>
-      </c>
     </row>
     <row r="35" xml:space="preserve">
       <c r="A35" t="str">
@@ -1775,12 +1569,6 @@
       <c r="J35" t="str">
         <v>village</v>
       </c>
-      <c r="K35">
-        <v>8</v>
-      </c>
-      <c r="L35">
-        <v>600</v>
-      </c>
     </row>
     <row r="36" xml:space="preserve">
       <c r="A36" t="str">
@@ -1814,12 +1602,6 @@
       <c r="J36" t="str">
         <v>village</v>
       </c>
-      <c r="K36">
-        <v>8</v>
-      </c>
-      <c r="L36">
-        <v>600</v>
-      </c>
     </row>
     <row r="37" xml:space="preserve">
       <c r="A37" t="str">
@@ -1853,12 +1635,6 @@
       <c r="J37" t="str">
         <v>village</v>
       </c>
-      <c r="K37">
-        <v>8</v>
-      </c>
-      <c r="L37">
-        <v>600</v>
-      </c>
     </row>
     <row r="38" xml:space="preserve">
       <c r="A38" t="str">
@@ -1892,12 +1668,6 @@
       <c r="J38" t="str">
         <v>village</v>
       </c>
-      <c r="K38">
-        <v>8</v>
-      </c>
-      <c r="L38">
-        <v>600</v>
-      </c>
     </row>
     <row r="39" xml:space="preserve">
       <c r="A39" t="str">
@@ -1931,12 +1701,6 @@
       <c r="J39" t="str">
         <v>village</v>
       </c>
-      <c r="K39">
-        <v>8</v>
-      </c>
-      <c r="L39">
-        <v>600</v>
-      </c>
     </row>
     <row r="40" xml:space="preserve">
       <c r="A40" t="str">
@@ -1970,12 +1734,6 @@
       <c r="J40" t="str">
         <v>village</v>
       </c>
-      <c r="K40">
-        <v>8</v>
-      </c>
-      <c r="L40">
-        <v>600</v>
-      </c>
     </row>
     <row r="41" xml:space="preserve">
       <c r="A41" t="str">
@@ -2009,12 +1767,6 @@
       <c r="J41" t="str">
         <v>city</v>
       </c>
-      <c r="K41">
-        <v>6</v>
-      </c>
-      <c r="L41">
-        <v>900</v>
-      </c>
     </row>
     <row r="42" xml:space="preserve">
       <c r="A42" t="str">
@@ -2048,12 +1800,6 @@
       <c r="J42" t="str">
         <v>city</v>
       </c>
-      <c r="K42">
-        <v>6</v>
-      </c>
-      <c r="L42">
-        <v>900</v>
-      </c>
     </row>
     <row r="43" xml:space="preserve">
       <c r="A43" t="str">
@@ -2087,15 +1833,9 @@
       <c r="J43" t="str">
         <v>village</v>
       </c>
-      <c r="K43">
-        <v>8</v>
-      </c>
-      <c r="L43">
-        <v>600</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L43"/>
+  <autoFilter ref="A1:J43"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:L43"/>
   </ignoredErrors>

</xml_diff>